<commit_message>
Actualización de datos: torneos de varios días unificados
Se unifican las fechas de eventos que estaban repartidos por día:
- Juegos de Integración Nikkei (marzo 2024): 4 filas -> 1 torneo.
- Torneo Día de Pa & Ma (julio 2025): 7 filas -> 1 torneo.
- XXI Torneo AOPCOOP (octubre 2024): 6 filas -> 1 torneo.

189 torneos, 714 jugadores, 225 equipos, 1.040 resultados (1.180 páginas).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/copas_y_torneos.xlsx
+++ b/data/raw/copas_y_torneos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\gateball\kantokeando-data\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB842DD0-6F67-42C3-80E1-9713BC04467E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3245F3C1-A9DF-49E7-A0FF-F7AF9FF244BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5079,7 +5079,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5099,6 +5099,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -9255,7 +9256,7 @@
       <c r="D136" t="s">
         <v>282</v>
       </c>
-      <c r="E136" s="13">
+      <c r="E136" s="15">
         <v>42106</v>
       </c>
       <c r="F136" s="13"/>
@@ -28441,7 +28442,7 @@
         <v>1255</v>
       </c>
       <c r="E785" s="5">
-        <v>45579</v>
+        <v>45578</v>
       </c>
       <c r="G785" s="9" t="s">
         <v>71</v>
@@ -28470,7 +28471,7 @@
         <v>1255</v>
       </c>
       <c r="E786" s="5">
-        <v>45580</v>
+        <v>45578</v>
       </c>
       <c r="G786" s="9" t="s">
         <v>71</v>
@@ -28499,7 +28500,7 @@
         <v>1255</v>
       </c>
       <c r="E787" s="5">
-        <v>45581</v>
+        <v>45578</v>
       </c>
       <c r="G787" s="9" t="s">
         <v>71</v>
@@ -28528,7 +28529,7 @@
         <v>1255</v>
       </c>
       <c r="E788" s="5">
-        <v>45582</v>
+        <v>45578</v>
       </c>
       <c r="G788" s="9" t="s">
         <v>71</v>
@@ -28557,7 +28558,7 @@
         <v>1255</v>
       </c>
       <c r="E789" s="5">
-        <v>45583</v>
+        <v>45578</v>
       </c>
       <c r="G789" s="9" t="s">
         <v>71</v>
@@ -28586,7 +28587,7 @@
         <v>1255</v>
       </c>
       <c r="E790" s="5">
-        <v>45584</v>
+        <v>45578</v>
       </c>
       <c r="G790" s="9" t="s">
         <v>71</v>
@@ -29920,7 +29921,7 @@
         <v>303</v>
       </c>
       <c r="E837" s="5">
-        <v>45369</v>
+        <v>45368</v>
       </c>
       <c r="G837" s="9" t="s">
         <v>71</v>
@@ -29949,7 +29950,7 @@
         <v>303</v>
       </c>
       <c r="E838" s="5">
-        <v>45370</v>
+        <v>45368</v>
       </c>
       <c r="G838" s="9" t="s">
         <v>71</v>
@@ -29978,7 +29979,7 @@
         <v>303</v>
       </c>
       <c r="E839" s="5">
-        <v>45371</v>
+        <v>45368</v>
       </c>
       <c r="G839" s="9" t="s">
         <v>71</v>
@@ -30007,7 +30008,7 @@
         <v>303</v>
       </c>
       <c r="E840" s="5">
-        <v>45372</v>
+        <v>45368</v>
       </c>
       <c r="G840" s="9" t="s">
         <v>71</v>
@@ -32121,7 +32122,7 @@
         <v>1443</v>
       </c>
       <c r="E916" s="5">
-        <v>45852</v>
+        <v>45851</v>
       </c>
       <c r="G916" t="s">
         <v>15</v>
@@ -32147,7 +32148,7 @@
         <v>1443</v>
       </c>
       <c r="E917" s="5">
-        <v>45853</v>
+        <v>45851</v>
       </c>
       <c r="G917" t="s">
         <v>15</v>
@@ -32173,7 +32174,7 @@
         <v>1443</v>
       </c>
       <c r="E918" s="5">
-        <v>45854</v>
+        <v>45851</v>
       </c>
       <c r="G918" t="s">
         <v>15</v>
@@ -32199,7 +32200,7 @@
         <v>1443</v>
       </c>
       <c r="E919" s="5">
-        <v>45855</v>
+        <v>45851</v>
       </c>
       <c r="G919" t="s">
         <v>15</v>
@@ -32225,7 +32226,7 @@
         <v>1443</v>
       </c>
       <c r="E920" s="5">
-        <v>45856</v>
+        <v>45851</v>
       </c>
       <c r="G920" t="s">
         <v>15</v>
@@ -32251,7 +32252,7 @@
         <v>1443</v>
       </c>
       <c r="E921" s="5">
-        <v>45857</v>
+        <v>45851</v>
       </c>
       <c r="G921" t="s">
         <v>15</v>
@@ -32277,7 +32278,7 @@
         <v>1443</v>
       </c>
       <c r="E922" s="5">
-        <v>45858</v>
+        <v>45851</v>
       </c>
       <c r="G922" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
Datos: alias de Aikokai y Johny Tsuhako, torneo reasignado a Torneo Club Aikokai en el Excel
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/copas_y_torneos.xlsx
+++ b/data/raw/copas_y_torneos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\gateball\kantokeando-data\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{767C59F6-0244-4F03-8AFF-562892B3321B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE30C624-6B90-4945-826B-BF3E52E8DFB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resultados" sheetId="1" r:id="rId1"/>
@@ -29836,7 +29836,7 @@
     </row>
     <row r="820" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C820" t="s">
-        <v>27</v>
+        <v>129</v>
       </c>
       <c r="D820" t="s">
         <v>1313</v>
@@ -29865,7 +29865,7 @@
     </row>
     <row r="821" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C821" t="s">
-        <v>27</v>
+        <v>129</v>
       </c>
       <c r="D821" t="s">
         <v>1313</v>
@@ -29894,7 +29894,7 @@
     </row>
     <row r="822" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C822" t="s">
-        <v>27</v>
+        <v>129</v>
       </c>
       <c r="D822" t="s">
         <v>1313</v>
@@ -29923,7 +29923,7 @@
     </row>
     <row r="823" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C823" t="s">
-        <v>27</v>
+        <v>129</v>
       </c>
       <c r="D823" t="s">
         <v>1313</v>
@@ -29952,7 +29952,7 @@
     </row>
     <row r="824" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C824" t="s">
-        <v>27</v>
+        <v>129</v>
       </c>
       <c r="D824" t="s">
         <v>1313</v>
@@ -29981,7 +29981,7 @@
     </row>
     <row r="825" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C825" t="s">
-        <v>27</v>
+        <v>129</v>
       </c>
       <c r="D825" t="s">
         <v>1313</v>
@@ -30010,7 +30010,7 @@
     </row>
     <row r="826" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C826" t="s">
-        <v>27</v>
+        <v>129</v>
       </c>
       <c r="D826" t="s">
         <v>1313</v>
@@ -30039,7 +30039,7 @@
     </row>
     <row r="827" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C827" t="s">
-        <v>27</v>
+        <v>129</v>
       </c>
       <c r="D827" t="s">
         <v>1313</v>

</xml_diff>

<commit_message>
Datos: corrección en el Excel (Torneo Club Sakura 2026) y JSON re-exportados
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/copas_y_torneos.xlsx
+++ b/data/raw/copas_y_torneos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\gateball\kantokeando-data\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E1EE6E5-F7C5-4A0D-93DD-6E5A5411C9BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A62F31FB-B13C-403E-AC98-877D5C952347}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resultados" sheetId="1" r:id="rId1"/>
@@ -35251,7 +35251,7 @@
         <v>2</v>
       </c>
       <c r="K1004" t="s">
-        <v>514</v>
+        <v>639</v>
       </c>
       <c r="L1004" t="s">
         <v>1603</v>

</xml_diff>

<commit_message>
Datos: 4 registros nuevos (XXVIII Campeonato Interno Amistoso - Jinnai) y JSON re-exportados
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/copas_y_torneos.xlsx
+++ b/data/raw/copas_y_torneos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\gateball\kantokeando-data\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A62F31FB-B13C-403E-AC98-877D5C952347}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{801F71AE-05BD-4BEB-9DB1-17853D6D06D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8241" uniqueCount="1712">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8245" uniqueCount="1712">
   <si>
     <t>id_torneo</t>
   </si>
@@ -5387,7 +5387,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5448,6 +5448,7 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -31569,6 +31570,9 @@
       <c r="B878" t="s">
         <v>137</v>
       </c>
+      <c r="C878" t="s">
+        <v>521</v>
+      </c>
       <c r="D878" t="s">
         <v>1397</v>
       </c>
@@ -31595,6 +31599,9 @@
       <c r="B879" t="s">
         <v>137</v>
       </c>
+      <c r="C879" t="s">
+        <v>521</v>
+      </c>
       <c r="D879" t="s">
         <v>1397</v>
       </c>
@@ -31621,6 +31628,9 @@
       <c r="B880" t="s">
         <v>137</v>
       </c>
+      <c r="C880" s="30" t="s">
+        <v>521</v>
+      </c>
       <c r="D880" t="s">
         <v>1397</v>
       </c>
@@ -31646,6 +31656,9 @@
     <row r="881" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B881" t="s">
         <v>137</v>
+      </c>
+      <c r="C881" t="s">
+        <v>521</v>
       </c>
       <c r="D881" t="s">
         <v>1397</v>

</xml_diff>